<commit_message>
Clarify lowercase preflight domain names
</commit_message>
<xml_diff>
--- a/spreadsheets/CRAMPACS_Governance_Master.xlsx
+++ b/spreadsheets/CRAMPACS_Governance_Master.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7874eb4965944b70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Matrix" sheetId="2" r:id="Rb8d8641eb83f47a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc Layers" sheetId="3" r:id="R8c28ce8c14244a94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Gates" sheetId="4" r:id="Rb863f7148df645cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gotchas" sheetId="5" r:id="R1f9843d1d19e4dc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preflight Checklist" sheetId="6" r:id="R38f25f2423bd4bd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Gate Tracker" sheetId="7" r:id="R9092c70f0de94171"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbcc31a42309d4c46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Matrix" sheetId="2" r:id="R4d2531a68e3b4991"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc Layers" sheetId="3" r:id="R76b0dc31fb104dcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Gates" sheetId="4" r:id="R68d0c0295e7244cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gotchas" sheetId="5" r:id="R707db8b45d3b4206"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preflight Checklist" sheetId="6" r:id="Rb42d6fdd15b1409e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Gate Tracker" sheetId="7" r:id="R96dbd032387f4810"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -262,10 +262,10 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
+        <x:v>Preflight</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
         <x:v>Full System</x:v>
-      </x:c>
-      <x:c r="B1" t="str">
-        <x:v>Preflight</x:v>
       </x:c>
       <x:c r="C1" t="str">
         <x:v>Domain</x:v>
@@ -285,10 +285,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
+        <x:v>crampacs-med</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
         <x:v>CRAMPACS-MED</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>crampacs-med</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>Medicine and clinical evidence</x:v>
@@ -308,10 +308,10 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
+        <x:v>crampacs-gen</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
         <x:v>CRAMPACS-GEN</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>crampacs-gen</x:v>
       </x:c>
       <x:c r="C3" t="str">
         <x:v>Genomics and omics</x:v>
@@ -331,10 +331,10 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
+        <x:v>crampacs-clim</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
         <x:v>CRAMPACS-CLIM</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
-        <x:v>crampacs-clim</x:v>
       </x:c>
       <x:c r="C4" t="str">
         <x:v>Climate and Earth systems</x:v>
@@ -354,10 +354,10 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
+        <x:v>crampacs-mat</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
         <x:v>CRAMPACS-MAT</x:v>
-      </x:c>
-      <x:c r="B5" t="str">
-        <x:v>crampacs-mat</x:v>
       </x:c>
       <x:c r="C5" t="str">
         <x:v>Materials science</x:v>
@@ -377,10 +377,10 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
+        <x:v>crampacs-eng</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
         <x:v>CRAMPACS-ENG</x:v>
-      </x:c>
-      <x:c r="B6" t="str">
-        <x:v>crampacs-eng</x:v>
       </x:c>
       <x:c r="C6" t="str">
         <x:v>Engineering reliability</x:v>
@@ -400,10 +400,10 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
+        <x:v>crampacs-fin</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
         <x:v>CRAMPACS-FIN</x:v>
-      </x:c>
-      <x:c r="B7" t="str">
-        <x:v>crampacs-fin</x:v>
       </x:c>
       <x:c r="C7" t="str">
         <x:v>Finance, fraud, and risk</x:v>
@@ -423,10 +423,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
+        <x:v>crampacs-cyb</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
         <x:v>CRAMPACS-CYB</x:v>
-      </x:c>
-      <x:c r="B8" t="str">
-        <x:v>crampacs-cyb</x:v>
       </x:c>
       <x:c r="C8" t="str">
         <x:v>Cybersecurity</x:v>
@@ -446,10 +446,10 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
+        <x:v>crampacs-ast</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
         <x:v>CRAMPACS-AST</x:v>
-      </x:c>
-      <x:c r="B9" t="str">
-        <x:v>crampacs-ast</x:v>
       </x:c>
       <x:c r="C9" t="str">
         <x:v>Astronomy and astrophysics</x:v>
@@ -469,10 +469,10 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
+        <x:v>crampacs-phy</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
         <x:v>CRAMPACS-PHY</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>crampacs-phy</x:v>
       </x:c>
       <x:c r="C10" t="str">
         <x:v>Physics and physical anomaly catalogs</x:v>

</xml_diff>

<commit_message>
Harden CRAMPACS assurance program
</commit_message>
<xml_diff>
--- a/spreadsheets/CRAMPACS_Governance_Master.xlsx
+++ b/spreadsheets/CRAMPACS_Governance_Master.xlsx
@@ -2,13 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbcc31a42309d4c46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Matrix" sheetId="2" r:id="R4d2531a68e3b4991"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc Layers" sheetId="3" r:id="R76b0dc31fb104dcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Gates" sheetId="4" r:id="R68d0c0295e7244cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gotchas" sheetId="5" r:id="R707db8b45d3b4206"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preflight Checklist" sheetId="6" r:id="Rb42d6fdd15b1409e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Gate Tracker" sheetId="7" r:id="R96dbd032387f4810"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5590febf090a42df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Matrix" sheetId="2" r:id="R9947316394a34e91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc Layers" sheetId="3" r:id="R51d75df5cf1945e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Gates" sheetId="4" r:id="R09fdeaaa556742aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Catalog" sheetId="5" r:id="Rde46a76c1cdb4d88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assurance Claims" sheetId="6" r:id="Re7502e02584345e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supervisor Questions" sheetId="7" r:id="R0874b90706264f5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Batteries" sheetId="8" r:id="R2e48b23adeb94767"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Scaffold" sheetId="9" r:id="R717615e641ea4a02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Registers" sheetId="10" r:id="R98d4dc84f816485b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPA Log" sheetId="11" r:id="R53d4edf3cf0c42af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gotchas" sheetId="12" r:id="Rd404b7032cd64fd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preflight Checklist" sheetId="13" r:id="R2243490557734915"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Gate Tracker" sheetId="14" r:id="R0eb6827d93934e4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -256,6 +263,501 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Register</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>Review status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>document_register.csv</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>document control, version, status, approval</x:v>
+      </x:c>
+      <x:c r="C2" t="str"/>
+      <x:c r="D2" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>control_evidence_register.csv</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>control-by-control evidence map</x:v>
+      </x:c>
+      <x:c r="C3" t="str"/>
+      <x:c r="D3" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>gate_review_record.csv</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>gate decisions, blockers, release holds</x:v>
+      </x:c>
+      <x:c r="C4" t="str"/>
+      <x:c r="D4" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>assurance_case_register.csv</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>claim, evidence, rebuttal, residual risk</x:v>
+      </x:c>
+      <x:c r="C5" t="str"/>
+      <x:c r="D5" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>deviation_capa_log.csv</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>deviation, containment, CAPA, effectiveness</x:v>
+      </x:c>
+      <x:c r="C6" t="str"/>
+      <x:c r="D6" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>decision_log.csv</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>authorized decision, tier, conditions, prohibited claims</x:v>
+      </x:c>
+      <x:c r="C7" t="str"/>
+      <x:c r="D7" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>risk_register.csv</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>active and residual risks</x:v>
+      </x:c>
+      <x:c r="C8" t="str"/>
+      <x:c r="D8" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>training_matrix.csv</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>role training and competency</x:v>
+      </x:c>
+      <x:c r="C9" t="str"/>
+      <x:c r="D9" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Deviation ID</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Study ID</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Severity</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>Affected controls</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>Description</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>Containment</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>Root cause</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>Corrective action</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>Preventive action</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>Due date</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>Verification</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>Effectiveness check date</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>Effectiveness result</x:v>
+      </x:c>
+      <x:c r="O1" t="str">
+        <x:v>Approver</x:v>
+      </x:c>
+      <x:c r="P1" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str"/>
+      <x:c r="B2" t="str"/>
+      <x:c r="C2" t="str"/>
+      <x:c r="D2" t="str"/>
+      <x:c r="E2" t="str"/>
+      <x:c r="F2" t="str"/>
+      <x:c r="G2" t="str"/>
+      <x:c r="H2" t="str"/>
+      <x:c r="I2" t="str"/>
+      <x:c r="J2" t="str"/>
+      <x:c r="K2" t="str"/>
+      <x:c r="L2" t="str"/>
+      <x:c r="M2" t="str"/>
+      <x:c r="N2" t="str"/>
+      <x:c r="O2" t="str"/>
+      <x:c r="P2" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Gotcha</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Symptom</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Fast sanity check</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>Coordinate drift</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>Coordinate changes names, units, or definitions across sources</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>Write the coordinate formula and units on one line</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>Tolerance creep</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Window widens after rows are seen</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>State tolerance source before scoring</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Null starvation</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Only positive anomalies are included</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Find nulls, exclusions, failed replications, non-events</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Duplicate evidence</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Rows trace to one raw data source</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Draw source-to-row dependence graph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Literature fashion</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Many sources inspect same coordinate because it is popular</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Add coordinate-fashion bias</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Time leakage</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Later knowledge shaped earlier-looking lock</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Compare lock date with source dates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Unit trap</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Alignment depends on hidden conversion</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Recompute normalized values from raw values</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>One-source collapse</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>Remove one source and result disappears</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Leave-one-source-out</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>Negative control failure</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Controls also recur</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>Strengthen null model</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>AI extraction drift</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>AI summary becomes data</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Trace each row to source evidence</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Item</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>Scope written</x:v>
+      </x:c>
+      <x:c r="B2" t="str"/>
+      <x:c r="C2" t="str"/>
+      <x:c r="D2" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>Coordinate sketch complete</x:v>
+      </x:c>
+      <x:c r="B3" t="str"/>
+      <x:c r="C3" t="str"/>
+      <x:c r="D3" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Source shortlist complete</x:v>
+      </x:c>
+      <x:c r="B4" t="str"/>
+      <x:c r="C4" t="str"/>
+      <x:c r="D4" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Nulls/non-events found</x:v>
+      </x:c>
+      <x:c r="B5" t="str"/>
+      <x:c r="C5" t="str"/>
+      <x:c r="D5" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Dependence scan complete</x:v>
+      </x:c>
+      <x:c r="B6" t="str"/>
+      <x:c r="C6" t="str"/>
+      <x:c r="D6" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Bias scan complete</x:v>
+      </x:c>
+      <x:c r="B7" t="str"/>
+      <x:c r="C7" t="str"/>
+      <x:c r="D7" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Sidecar metrics run</x:v>
+      </x:c>
+      <x:c r="B8" t="str"/>
+      <x:c r="C8" t="str"/>
+      <x:c r="D8" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>Decision written</x:v>
+      </x:c>
+      <x:c r="B9" t="str"/>
+      <x:c r="C9" t="str"/>
+      <x:c r="D9" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Gate</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>Evidence link</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>G0 Charter</x:v>
+      </x:c>
+      <x:c r="B2" t="str"/>
+      <x:c r="C2" t="str"/>
+      <x:c r="D2" t="str"/>
+      <x:c r="E2" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>G1 Coordinate Lock</x:v>
+      </x:c>
+      <x:c r="B3" t="str"/>
+      <x:c r="C3" t="str"/>
+      <x:c r="D3" t="str"/>
+      <x:c r="E3" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>G2 Source Universe</x:v>
+      </x:c>
+      <x:c r="B4" t="str"/>
+      <x:c r="C4" t="str"/>
+      <x:c r="D4" t="str"/>
+      <x:c r="E4" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>G3 Row Integrity</x:v>
+      </x:c>
+      <x:c r="B5" t="str"/>
+      <x:c r="C5" t="str"/>
+      <x:c r="D5" t="str"/>
+      <x:c r="E5" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>G4 Dependence and Bias</x:v>
+      </x:c>
+      <x:c r="B6" t="str"/>
+      <x:c r="C6" t="str"/>
+      <x:c r="D6" t="str"/>
+      <x:c r="E6" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>G5 Statistical Method</x:v>
+      </x:c>
+      <x:c r="B7" t="str"/>
+      <x:c r="C7" t="str"/>
+      <x:c r="D7" t="str"/>
+      <x:c r="E7" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>G6 Reproducibility</x:v>
+      </x:c>
+      <x:c r="B8" t="str"/>
+      <x:c r="C8" t="str"/>
+      <x:c r="D8" t="str"/>
+      <x:c r="E8" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>G7 Release</x:v>
+      </x:c>
+      <x:c r="B9" t="str"/>
+      <x:c r="C9" t="str"/>
+      <x:c r="D9" t="str"/>
+      <x:c r="E9" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -317,7 +819,7 @@
         <x:v>Genomics and omics</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>locus; variant; gene; pathway; cell type; expression threshold</x:v>
+        <x:v>locus; variant; gene; pathway; cell type; tissue; expression threshold; perturbation</x:v>
       </x:c>
       <x:c r="E3" t="str">
         <x:v>failed replications; non-significant loci; negative functional assays; tested pathways not enriched</x:v>
@@ -340,7 +842,7 @@
         <x:v>Climate and Earth systems</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>latitude; longitude; depth; pressure level; season; climate mode</x:v>
+        <x:v>latitude; longitude; depth; pressure level; season; climate mode; threshold; basin</x:v>
       </x:c>
       <x:c r="E4" t="str">
         <x:v>comparable regions without anomaly; model runs without recurrence; negative attribution studies</x:v>
@@ -386,7 +888,7 @@
         <x:v>Engineering reliability</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>load; vibration frequency; temperature; firmware version; supplier lot; cycle count</x:v>
+        <x:v>load; vibration frequency; temperature; firmware version; supplier lot; cycle count; failure mode</x:v>
       </x:c>
       <x:c r="E6" t="str">
         <x:v>units exposed without failure; passed qualification tests; lots with no anomaly; sensor streams without recurrence</x:v>
@@ -409,7 +911,7 @@
         <x:v>Finance, fraud, and risk</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>asset; tenor; counterparty; time window; transaction velocity; network position</x:v>
+        <x:v>asset; tenor; counterparty; time window; transaction velocity; network position; model threshold</x:v>
       </x:c>
       <x:c r="E7" t="str">
         <x:v>cleared alerts; comparable accounts without event; backtests with no breach; control portfolios</x:v>
@@ -432,7 +934,7 @@
         <x:v>Cybersecurity</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>CVE; ATT&amp;CK technique; port; protocol; endpoint class; time-to-exploit</x:v>
+        <x:v>CVE; ATT&amp;CK technique; port; protocol; endpoint class; time-to-exploit; detection rule</x:v>
       </x:c>
       <x:c r="E8" t="str">
         <x:v>exposed assets not exploited; rules with no hits; scanned vulnerabilities not exploited; false positives</x:v>
@@ -455,7 +957,7 @@
         <x:v>Astronomy and astrophysics</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>sky coordinate; redshift; wavelength; period; phase; cadence</x:v>
+        <x:v>sky coordinate; redshift; wavelength; period; phase; cadence; source class</x:v>
       </x:c>
       <x:c r="E9" t="str">
         <x:v>follow-up non-detections; survey fields with no event; searched spectral windows with no feature</x:v>
@@ -478,10 +980,10 @@
         <x:v>Physics and physical anomaly catalogs</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>mass; energy; frequency; redshift; coupling; cross section</x:v>
+        <x:v>mass; energy; frequency; redshift; coupling; cross section; decay channel; event topology</x:v>
       </x:c>
       <x:c r="E10" t="str">
-        <x:v>null searches; exclusion contours; control regions; sidebands; failed replications</x:v>
+        <x:v>null searches; exclusion contours; control regions; sidebands; non-detections; failed replications</x:v>
       </x:c>
       <x:c r="F10" t="str">
         <x:v>look-elsewhere effect; theory-fashion clustering; shared detector pipelines; plot digitization error</x:v>
@@ -538,7 +1040,7 @@
         <x:v>1-2 day triage and seed artifacts</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>preflight policy and templates</x:v>
+        <x:v>preflight policy, preflight templates, domain packs</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -549,10 +1051,10 @@
         <x:v>Gotchas</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Fast failure-mode checks</x:v>
+        <x:v>Fast failure-mode checks and stop signs</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>gotcha guide and printouts</x:v>
+        <x:v>gotcha guide, field printouts</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -560,13 +1062,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Standards</x:v>
+        <x:v>Program standards</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Governance, quality gates, document control</x:v>
+        <x:v>Governance, quality gates, document control, release authority, CAPA</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>standards policy</x:v>
+        <x:v>program operating manual, control catalog, document control, release RACI, gate map, CAPA procedure</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -580,7 +1082,7 @@
         <x:v>Coordinate ontology, nulls, dependence, bias, claim tiers</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>methodology policy</x:v>
+        <x:v>methodology policy, protocol template</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -594,7 +1096,7 @@
         <x:v>Field-specific adaptation</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>domain overlays and packs</x:v>
+        <x:v>domain overlays, domain packs, field printouts</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -605,10 +1107,10 @@
         <x:v>Data contracts</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>Structured tables and stable IDs</x:v>
+        <x:v>Structured tables, stable IDs, register schemas</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>templates</x:v>
+        <x:v>templates, register data dictionary, package scaffold</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -622,7 +1124,7 @@
         <x:v>Cross-unit reproducibility and unit integrity</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>checksum policy</x:v>
+        <x:v>checksum policy, reproducibility binder</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -633,7 +1135,7 @@
         <x:v>Sidecar metrics</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>Package readiness and blockers</x:v>
+        <x:v>Package readiness, binder coverage, blockers</x:v>
       </x:c>
       <x:c r="D10" t="str">
         <x:v>sidecar runner</x:v>
@@ -647,10 +1149,10 @@
         <x:v>Full SOP</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>End-to-end study execution</x:v>
+        <x:v>End-to-end study execution and evidence package assembly</x:v>
       </x:c>
       <x:c r="D11" t="str">
-        <x:v>program SOP and protocol template</x:v>
+        <x:v>program SOP, evidence package spec, assurance case, decision memo</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -658,13 +1160,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Regulatory</x:v>
+        <x:v>Regulatory and deployment</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>Pair with domain controls</x:v>
+        <x:v>Safety supervisor review, audit, validation, training, regulated deployment</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>domain addenda</x:v>
+        <x:v>supervisor packet, audit procedure, validation plan, training plan, regulated addendum, deployment playbook, 90-day roadmap</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -703,68 +1205,90 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>Protocol</x:v>
+        <x:v>G0 Charter</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>Study charter, role assignment, protocol, candidate registry</x:v>
+        <x:v>decision statement, assurance level, roles, intended use, prohibited use</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Before extraction</x:v>
+        <x:v>Before protocol lock</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Extraction</x:v>
+        <x:v>G1 Coordinate Lock</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Source flow, exclusions, row provenance, extraction confidence</x:v>
+        <x:v>coordinate ontology, candidate registry, tolerance basis, transform rules, negative controls</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>Before normalization</x:v>
+        <x:v>Before source scoring</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Normalization</x:v>
+        <x:v>G2 Source Universe</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>Raw values preserved, transforms registered, uncertainty assigned</x:v>
+        <x:v>search strategy, source catalog, source flow, exclusions, null search</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Before analysis</x:v>
+        <x:v>Before extraction closeout</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Independence and bias</x:v>
+        <x:v>G3 Row Integrity</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Independence grades, bias review, missing evidence, weights</x:v>
+        <x:v>raw rows, source trace, extraction confidence, review status, quarantine log</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Before scoring</x:v>
+        <x:v>Before normalization closeout</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Statistical</x:v>
+        <x:v>G4 Dependence and Bias</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Primary statistic, null model, global correction, sensitivities</x:v>
+        <x:v>evidence-family map, independence grades, bias table, missing-evidence memo, weights</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>Before reporting</x:v>
+        <x:v>Before analysis</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Release</x:v>
+        <x:v>G5 Statistical Method</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Repro capsule, red team, signoff, claim language</x:v>
+        <x:v>primary statistic, null model, multiplicity correction, negative controls, sensitivity plan</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Before external use</x:v>
+        <x:v>Before reporting</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>G6 Reproducibility</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>checksums, environment, run script, output hashes, clean-run report</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Before release review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>G7 Release</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>assurance case, red-team findings, decision memo, evidence tier, claim-language approval</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Before external or operational use</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -778,123 +1302,282 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>Gotcha</x:v>
+        <x:v>Control ID</x:v>
       </x:c>
       <x:c r="B1" t="str">
-        <x:v>Symptom</x:v>
+        <x:v>Control</x:v>
       </x:c>
       <x:c r="C1" t="str">
-        <x:v>Fast sanity check</x:v>
+        <x:v>Objective</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>Evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>Coordinate drift</x:v>
+        <x:v>GOV-01</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>Coordinate changes names, units, or definitions across sources</x:v>
+        <x:v>Decision authority assigned</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Write the coordinate formula and units on one line</x:v>
+        <x:v>Prevent ownerless decisions</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>charter, role assignment, decision memo</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Tolerance creep</x:v>
+        <x:v>GOV-02</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Window widens after rows are seen</x:v>
+        <x:v>Assurance level declared</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>State tolerance source before scoring</x:v>
+        <x:v>Prevent lowercase work being treated as full assurance</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>charter, report title</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Null starvation</x:v>
+        <x:v>DOC-02</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>Only positive anomalies are included</x:v>
+        <x:v>Protocol lock</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Find nulls, exclusions, failed replications, non-events</x:v>
+        <x:v>Prevent post-hoc method changes</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>protocol hash, lock timestamp</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Duplicate evidence</x:v>
+        <x:v>COORD-01</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Rows trace to one raw data source</x:v>
+        <x:v>Coordinate definition</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Draw source-to-row dependence graph</x:v>
+        <x:v>Prevent vague or mobile target coordinates</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>coordinate ontology</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Literature fashion</x:v>
+        <x:v>COORD-02</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Many sources inspect same coordinate because it is popular</x:v>
+        <x:v>Tolerance justification</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>Add coordinate-fashion bias</x:v>
+        <x:v>Prevent tolerance creep</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>candidate registry</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Time leakage</x:v>
+        <x:v>SRC-02</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Later knowledge shaped earlier-looking lock</x:v>
+        <x:v>Null/non-event search</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Compare lock date with source dates</x:v>
+        <x:v>Prevent positive-only evidence</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>source catalog, null row count</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Unit trap</x:v>
+        <x:v>ROW-01</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Alignment depends on hidden conversion</x:v>
+        <x:v>Row provenance</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>Recompute normalized values from raw values</x:v>
+        <x:v>Ensure every row traces to source</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>raw row table</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>One-source collapse</x:v>
+        <x:v>ROW-02</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>Remove one source and result disappears</x:v>
+        <x:v>Raw/normalized separation</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>Leave-one-source-out</x:v>
+        <x:v>Prevent unit and transform overwrites</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>raw and normalized tables</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>Negative control failure</x:v>
+        <x:v>IND-01</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>Controls also recur</x:v>
+        <x:v>Evidence-family map</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>Strengthen null model</x:v>
+        <x:v>Prevent duplicate evidence multiplication</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>independence groups</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>AI extraction drift</x:v>
+        <x:v>BIAS-01</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>AI summary becomes data</x:v>
+        <x:v>Missing-evidence assessment</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>Trace each row to source evidence</x:v>
+        <x:v>Identify inaccessible or unpublished nulls</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>missing-evidence memo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>STAT-02</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>Null model specification</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Make the test basis explicit</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>null model spec</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>STAT-03</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>Global correction</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Control look-elsewhere and multiplicity</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>result table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>STAT-04</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>Sensitivity tests</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Identify fragility</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>sensitivity results</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>REPRO-01</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>Checksum manifest</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Detect silent file drift</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>manifest and hashes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>REPRO-03</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Clean reproduction</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Verify package can be rerun</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>reproducibility report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>REL-01</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>Evidence tier assignment</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>Prevent overclaiming</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>evidence tier table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>REL-02</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>Claim language approval</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>Prevent unsupported conclusions</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>signed report review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>CAPA-01</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>Deviation handling</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>Track failures and repairs</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>deviation/CAPA log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>TRAIN-01</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Role training</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Ensure operators know controls</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>training matrix</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -908,81 +1591,171 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>Item</x:v>
+        <x:v>Claim ID</x:v>
       </x:c>
       <x:c r="B1" t="str">
-        <x:v>Status</x:v>
+        <x:v>Claim</x:v>
       </x:c>
       <x:c r="C1" t="str">
-        <x:v>Owner</x:v>
+        <x:v>Required evidence</x:v>
       </x:c>
       <x:c r="D1" t="str">
-        <x:v>Notes</x:v>
+        <x:v>Common rebuttal</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>Scope written</x:v>
-      </x:c>
-      <x:c r="B2" t="str"/>
-      <x:c r="C2" t="str"/>
-      <x:c r="D2" t="str"/>
+        <x:v>AC-01</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>Coordinate was pre-specified</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>protocol hash, candidate registry</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>coordinate moved after rows were known</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Coordinate sketch complete</x:v>
-      </x:c>
-      <x:c r="B3" t="str"/>
-      <x:c r="C3" t="str"/>
-      <x:c r="D3" t="str"/>
+        <x:v>AC-02</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Source universe was not cherry-picked</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>search log, source flow</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>null sources omitted</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Source shortlist complete</x:v>
-      </x:c>
-      <x:c r="B4" t="str"/>
-      <x:c r="C4" t="str"/>
-      <x:c r="D4" t="str"/>
+        <x:v>AC-03</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Rows are traceable and correctly extracted</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>row table, source references</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>AI or analyst inferred values incorrectly</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Nulls/non-events found</x:v>
-      </x:c>
-      <x:c r="B5" t="str"/>
-      <x:c r="C5" t="str"/>
-      <x:c r="D5" t="str"/>
+        <x:v>AC-04</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Units and transforms are controlled</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>raw/normalized split, transform registry</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>hidden conversion created cluster</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Dependence scan complete</x:v>
-      </x:c>
-      <x:c r="B6" t="str"/>
-      <x:c r="C6" t="str"/>
-      <x:c r="D6" t="str"/>
+        <x:v>AC-05</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Dependence is modeled or controlled</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>evidence-family map, weights</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>duplicate evidence counted independently</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Bias scan complete</x:v>
-      </x:c>
-      <x:c r="B7" t="str"/>
-      <x:c r="C7" t="str"/>
-      <x:c r="D7" t="str"/>
+        <x:v>AC-06</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Missing evidence and bias are assessed</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>bias table, missing-evidence memo</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>reporting bias explains cluster</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Sidecar metrics run</x:v>
-      </x:c>
-      <x:c r="B8" t="str"/>
-      <x:c r="C8" t="str"/>
-      <x:c r="D8" t="str"/>
+        <x:v>AC-07</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Null model is fit for purpose</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>null spec, negative controls</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>null is too weak</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Decision written</x:v>
-      </x:c>
-      <x:c r="B9" t="str"/>
-      <x:c r="C9" t="str"/>
-      <x:c r="D9" t="str"/>
+        <x:v>AC-08</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>Multiple testing is addressed</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>global correction</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>local result is look-elsewhere artifact</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>AC-09</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Result is robust enough for tier</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>sensitivity tests</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>one source drives result</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>AC-10</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>Package is reproducible</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>checksums, clean run</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>output cannot be recreated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>AC-11</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>Claim language matches evidence</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>evidence tier, approved report</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>report overstates causality</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -995,74 +1768,396 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>Gate</x:v>
+        <x:v>No.</x:v>
       </x:c>
       <x:c r="B1" t="str">
-        <x:v>Status</x:v>
+        <x:v>Question</x:v>
       </x:c>
       <x:c r="C1" t="str">
-        <x:v>Owner</x:v>
+        <x:v>Answer</x:v>
       </x:c>
       <x:c r="D1" t="str">
         <x:v>Evidence link</x:v>
       </x:c>
       <x:c r="E1" t="str">
-        <x:v>Notes</x:v>
+        <x:v>Open risk</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>Protocol</x:v>
-      </x:c>
-      <x:c r="B2" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>What coordinate is being tested?</x:v>
+      </x:c>
       <x:c r="C2" t="str"/>
       <x:c r="D2" t="str"/>
       <x:c r="E2" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Extraction</x:v>
-      </x:c>
-      <x:c r="B3" t="str"/>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Was it locked before scoring?</x:v>
+      </x:c>
       <x:c r="C3" t="str"/>
       <x:c r="D3" t="str"/>
       <x:c r="E3" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Normalization</x:v>
-      </x:c>
-      <x:c r="B4" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>What nulls or non-events were included?</x:v>
+      </x:c>
       <x:c r="C4" t="str"/>
       <x:c r="D4" t="str"/>
       <x:c r="E4" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Independence and bias</x:v>
-      </x:c>
-      <x:c r="B5" t="str"/>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>What evidence is duplicated or dependent?</x:v>
+      </x:c>
       <x:c r="C5" t="str"/>
       <x:c r="D5" t="str"/>
       <x:c r="E5" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Statistical</x:v>
-      </x:c>
-      <x:c r="B6" t="str"/>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>What bias could create the pattern?</x:v>
+      </x:c>
       <x:c r="C6" t="str"/>
       <x:c r="D6" t="str"/>
       <x:c r="E6" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Release</x:v>
-      </x:c>
-      <x:c r="B7" t="str"/>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>What negative control was used?</x:v>
+      </x:c>
       <x:c r="C7" t="str"/>
       <x:c r="D7" t="str"/>
       <x:c r="E7" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>What would make us stop believing the recurrence?</x:v>
+      </x:c>
+      <x:c r="C8" t="str"/>
+      <x:c r="D8" t="str"/>
+      <x:c r="E8" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>Can the package be reproduced?</x:v>
+      </x:c>
+      <x:c r="C9" t="str"/>
+      <x:c r="D9" t="str"/>
+      <x:c r="E9" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>What action is being requested?</x:v>
+      </x:c>
+      <x:c r="C10" t="str"/>
+      <x:c r="D10" t="str"/>
+      <x:c r="E10" t="str"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>What claim is explicitly prohibited?</x:v>
+      </x:c>
+      <x:c r="C11" t="str"/>
+      <x:c r="D11" t="str"/>
+      <x:c r="E11" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Battery</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Name</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Test condition</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>Pass condition</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>Known negative</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>Recurrence should not exist</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>No false high-confidence recurrence</x:v>
+      </x:c>
+      <x:c r="E2" t="str"/>
+      <x:c r="F2" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Synthetic planted cluster</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>Known recurrence is injected</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>Detects planted recurrence under registered statistic</x:v>
+      </x:c>
+      <x:c r="E3" t="str"/>
+      <x:c r="F3" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Duplicate-evidence trap</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Many rows derive from one source family</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Down-weights or collapses duplicates</x:v>
+      </x:c>
+      <x:c r="E4" t="str"/>
+      <x:c r="F4" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Missing-null trap</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Nulls are hidden until audit</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>Flags missing evidence and demotes/holds</x:v>
+      </x:c>
+      <x:c r="E5" t="str"/>
+      <x:c r="F5" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Unit-conversion trap</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Mixed units/reference systems</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>Raw/normalized audit catches drift</x:v>
+      </x:c>
+      <x:c r="E6" t="str"/>
+      <x:c r="F6" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Inter-rater reliability</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Independent reviewers grade same sample</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>Disagreements measured and adjudicated</x:v>
+      </x:c>
+      <x:c r="E7" t="str"/>
+      <x:c r="F7" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Binder</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Minimum records</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>00_charter</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>decision, roles, intended use, prohibited use, constraints</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>study_charter.md; role_assignment.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>01_protocol_lock</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>protocol, candidate registry, amendment control</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>protocol.md; candidate_coordinate_registry.csv; amendment_log.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>02_sources</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>search strategy, source catalog, source flow</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>search_strategy.md; source_catalog.csv; source_flow.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>03_extraction</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>raw rows and extraction review</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>anomaly_rows_raw.csv; extraction_notes.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>04_coordinate_normalization</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>transforms, normalized rows, unit audit</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>coordinate_transform_registry.csv; normalized_rows.csv; unit_conversion_audit.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>05_dependence_bias</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>independence, bias, missing evidence</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>independence_groups.csv; bias_assessment.csv; missing_evidence_assessment.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>06_statistics</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>analysis plan, null model, result, controls, sensitivities</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>statistical_analysis_plan.md; null_model_runs.csv; analysis_result.csv; negative_controls.md; sensitivity_results.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>07_reproducibility</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>checksums, environment, run instructions, clean run</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>checksum_manifest.csv; environment_record.md; run_instructions.md; clean_run_report.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>08_assurance_case</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>claims, rebuttals, residual risk</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>assurance_case.md; assurance_case_register.csv; risk_register.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>09_review_and_release</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>gate review, audit, decision, release signoff</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>gate_review_record.csv; audit_report.md; decision_memo.md; claim_language_approval.md; release_signoff.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>registers</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>package-level governance registers</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>document; control; gate; assurance; CAPA; decision; risk; training</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add CRAMPACS brand and training system
</commit_message>
<xml_diff>
--- a/spreadsheets/CRAMPACS_Governance_Master.xlsx
+++ b/spreadsheets/CRAMPACS_Governance_Master.xlsx
@@ -2,20 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5590febf090a42df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Matrix" sheetId="2" r:id="R9947316394a34e91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc Layers" sheetId="3" r:id="R51d75df5cf1945e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Gates" sheetId="4" r:id="R09fdeaaa556742aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Catalog" sheetId="5" r:id="Rde46a76c1cdb4d88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assurance Claims" sheetId="6" r:id="Re7502e02584345e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supervisor Questions" sheetId="7" r:id="R0874b90706264f5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Batteries" sheetId="8" r:id="R2e48b23adeb94767"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Scaffold" sheetId="9" r:id="R717615e641ea4a02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Registers" sheetId="10" r:id="R98d4dc84f816485b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPA Log" sheetId="11" r:id="R53d4edf3cf0c42af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gotchas" sheetId="12" r:id="Rd404b7032cd64fd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preflight Checklist" sheetId="13" r:id="R2243490557734915"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Gate Tracker" sheetId="14" r:id="R0eb6827d93934e4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf30773c6283e4da9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Matrix" sheetId="2" r:id="R47f1038f2fc445fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc Layers" sheetId="3" r:id="Re5bed857ba1b4da8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Gates" sheetId="4" r:id="R242e5c977c984c85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Catalog" sheetId="5" r:id="R23c0d6c106944759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assurance Claims" sheetId="6" r:id="R4f81538321504341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supervisor Questions" sheetId="7" r:id="R9fd8a3e7f41e4b5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Batteries" sheetId="8" r:id="R1d6131326589498c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Scaffold" sheetId="9" r:id="R02687cb35bad4280"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Registers" sheetId="10" r:id="Rbea8b54329d7489b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Controls" sheetId="11" r:id="R077b9c6fe61944d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training Paths" sheetId="12" r:id="R960d177f00d24501"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework Patterns" sheetId="13" r:id="Rf7da47e387484a64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPA Log" sheetId="14" r:id="R5f4b8738c57945e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gotchas" sheetId="15" r:id="Rc07049a8045b4239"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preflight Checklist" sheetId="16" r:id="R67be294b565e40fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Gate Tracker" sheetId="17" r:id="R57b1499377d74442"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -372,6 +375,316 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
+        <x:v>Control</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>Assurance boundary</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>Every artifact states whether it is crampacs-* or CRAMPACS-*</x:v>
+      </x:c>
+      <x:c r="C2" t="str"/>
+      <x:c r="D2" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>Claim boundary</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Every release-facing artifact states what CRAMPACS does not prove</x:v>
+      </x:c>
+      <x:c r="C3" t="str"/>
+      <x:c r="D3" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Decision language</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Approve, approve_with_limits, hold, demote, reject, stop, emergency_parallel_action</x:v>
+      </x:c>
+      <x:c r="C4" t="str"/>
+      <x:c r="D4" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Severity language</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Critical, Major, Minor, Observation</x:v>
+      </x:c>
+      <x:c r="C5" t="str"/>
+      <x:c r="D5" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Stop signs</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Preflight and full package stop rules are easy to find</x:v>
+      </x:c>
+      <x:c r="C6" t="str"/>
+      <x:c r="D6" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Evidence names</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Required evidence uses concrete file, register, or binder names</x:v>
+      </x:c>
+      <x:c r="C7" t="str"/>
+      <x:c r="D7" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Domain humility</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Domain claims are restrained and require domain-standard confirmation</x:v>
+      </x:c>
+      <x:c r="C8" t="str"/>
+      <x:c r="D8" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Track</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Audience</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Duration</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>Executive briefing</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>Sponsor, agency lead, director</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>60 minutes</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>adoption decision and pilot scope</x:v>
+      </x:c>
+      <x:c r="E2" t="str"/>
+      <x:c r="F2" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>Supervisor orientation</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Safety supervisor, risk owner, program officer</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>2 hours</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>approval, hold, demote, reject literacy</x:v>
+      </x:c>
+      <x:c r="E3" t="str"/>
+      <x:c r="F3" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Preflight workshop</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Analyst, domain reviewer, project lead</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>1 day</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>completed mock crampacs-* preflight</x:v>
+      </x:c>
+      <x:c r="E4" t="str"/>
+      <x:c r="F4" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Practitioner course</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Data scientist, evidence reviewer, auditor</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>3 days</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>full package walkthrough and gate practice</x:v>
+      </x:c>
+      <x:c r="E5" t="str"/>
+      <x:c r="F5" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Instructor course</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Internal trainer, quality lead</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>2 days after practitioner course</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>teach-back and scoring consistency</x:v>
+      </x:c>
+      <x:c r="E6" t="str"/>
+      <x:c r="F6" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Framework</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Pattern</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>CRAMPACS adoption</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>PRISMA</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>Checklist plus flow diagrams</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>Use checklists, printouts, and package flow</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>Cochrane</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Missing-evidence risk</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>Treat nulls, non-events, and missing evidence as release issues</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>GRADE</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Separate certainty and recommendation</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Separate evidence tier from supervisor decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>ISO quality management</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Process, evidence-based decisions, improvement</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Use owners, registers, CAPA, and review cadence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>NIST CSF</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Core, examples, references, tiers</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Keep a small core with implementation examples and maturity levels</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>NIST AI RMF</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Framework plus playbook</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Pair principles with teachable actions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>NASA systems engineering</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Lifecycle reviews</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Use G0-G7 as lifecycle gates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>FDA quality systems</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>Quality model plus regulatory boundary</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Add regulated controls without claiming automatic compliance</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
         <x:v>Deviation ID</x:v>
       </x:c>
       <x:c r="B1" t="str">
@@ -443,7 +756,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -573,7 +886,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -660,7 +973,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>

</xml_diff>

<commit_message>
Add CRAMPACS CLI trust gate system
</commit_message>
<xml_diff>
--- a/spreadsheets/CRAMPACS_Governance_Master.xlsx
+++ b/spreadsheets/CRAMPACS_Governance_Master.xlsx
@@ -2,23 +2,26 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf30773c6283e4da9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Matrix" sheetId="2" r:id="R47f1038f2fc445fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc Layers" sheetId="3" r:id="Re5bed857ba1b4da8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Gates" sheetId="4" r:id="R242e5c977c984c85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Catalog" sheetId="5" r:id="R23c0d6c106944759"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assurance Claims" sheetId="6" r:id="R4f81538321504341"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supervisor Questions" sheetId="7" r:id="R9fd8a3e7f41e4b5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Batteries" sheetId="8" r:id="R1d6131326589498c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Scaffold" sheetId="9" r:id="R02687cb35bad4280"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Registers" sheetId="10" r:id="Rbea8b54329d7489b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Controls" sheetId="11" r:id="R077b9c6fe61944d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training Paths" sheetId="12" r:id="R960d177f00d24501"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework Patterns" sheetId="13" r:id="Rf7da47e387484a64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPA Log" sheetId="14" r:id="R5f4b8738c57945e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gotchas" sheetId="15" r:id="Rc07049a8045b4239"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preflight Checklist" sheetId="16" r:id="R67be294b565e40fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Gate Tracker" sheetId="17" r:id="R57b1499377d74442"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1fbadaa43d374e6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Matrix" sheetId="2" r:id="R59609d8599754375"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc Layers" sheetId="3" r:id="Rf26cb0a992bc4168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Gates" sheetId="4" r:id="R2ac92f9085fe470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Catalog" sheetId="5" r:id="R69171ac24a8b4670"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assurance Claims" sheetId="6" r:id="R1b5ac12ed8284de3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supervisor Questions" sheetId="7" r:id="R75c85e2153bf4dcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Batteries" sheetId="8" r:id="R4ea94fd317304e55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Scaffold" sheetId="9" r:id="R5c9655f16d224db1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Registers" sheetId="10" r:id="R17843f206f044dc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Controls" sheetId="11" r:id="Rbe618cdfbc1e4c03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training Paths" sheetId="12" r:id="R9274ed5b49c84203"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework Patterns" sheetId="13" r:id="R4d440d8d9f1a4d2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trust States" sheetId="14" r:id="R785d7fb6503b4b5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reliance Levels" sheetId="15" r:id="Radf4ce34c02a4873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trust Checkpoints" sheetId="16" r:id="Ra153911296c946cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPA Log" sheetId="17" r:id="R826c20525dc943a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gotchas" sheetId="18" r:id="R1ef196bbfbb041a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preflight Checklist" sheetId="19" r:id="R2c2a55203533489d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Gate Tracker" sheetId="20" r:id="R7a9349df3d754608"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -250,7 +253,7 @@
         <x:v>Layer count</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -364,6 +367,16 @@
       <x:c r="C9" t="str"/>
       <x:c r="D9" t="str"/>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>trust_debt_register.csv</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>unresolved trust gaps and release impact</x:v>
+      </x:c>
+      <x:c r="C10" t="str"/>
+      <x:c r="D10" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -680,6 +693,352 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Trust state</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Meaning</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Reliance rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>draft</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>work has started but is not checked</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>do not rely</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>unchecked</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>artifact exists but no reviewer has accepted it</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>do not rely</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>checked_with_limits</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>reviewed, but known limits remain</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>rely only within stated limits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>reviewed and accepted for current gate</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>rely within current evidence tier</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>blocked</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>has a defect that prevents promotion or release</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>do not promote</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>superseded</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>replaced by a newer artifact</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>retain but do not use</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>quarantined</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>retained for traceability but excluded from scoring or release</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>do not use as evidence</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Package state</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Trustworthy for</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Not trustworthy for</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>idea sketch</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>conversation and scoping</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>CRAMPACS claim, preflight decision, operational decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>crampacs-* checked</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>continue, hold, stop, or full-study escalation</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>domain conclusion, full assurance, external claim</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>CRAMPACS-* scaffold</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>organizing work</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>evidence reliance or release</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>CRAMPACS-* gate-accepted</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>advancing to the next gate</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>release unless G7 is complete</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>CRAMPACS-* release-ready</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>decision support within assigned evidence tier</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>proof of causality or regulatory compliance by itself</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>externally validated</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>stronger prioritization and process confidence</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>domain proof unless domain-standard confirmation is complete</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Checkpoint</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Package point</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Main honesty risk</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>Minimum review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>T0</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>package start</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>unclear purpose or hidden intended use</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>decision owner, intended use, prohibited use</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>T1</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>coordinate proposed</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>coordinate drift or tolerance creep</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>coordinate, units, tolerance, forbidden changes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>T2</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>sources drafted</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>positive-only evidence</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>source roles, null search, exclusions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>T3</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>rows extracted</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>source trace or AI-summary drift</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>source links, raw values, extraction confidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>T4</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>normalization drafted</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>hidden unit conversion</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>raw/normalized separation, transform review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>T5</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>dependence and bias drafted</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>duplicate evidence counted independently</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>evidence-family map, missing-evidence risk</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>T6</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>statistics planned</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>statistic shopping or weak null</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>locked statistic, null model, multiplicity plan</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>T7</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>results generated</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>local result overclaimed</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>global correction, sensitivities, negative controls</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>T8</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>report drafted</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>claim exceeds evidence tier</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>claim trace matrix, prohibited claims</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>T9</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>release review</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>unknown trust state</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>trust status summary, sidecar, open CAPA</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -756,7 +1115,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -886,7 +1245,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -967,104 +1326,6 @@
       <x:c r="B9" t="str"/>
       <x:c r="C9" t="str"/>
       <x:c r="D9" t="str"/>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" t="str">
-        <x:v>Gate</x:v>
-      </x:c>
-      <x:c r="B1" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="C1" t="str">
-        <x:v>Owner</x:v>
-      </x:c>
-      <x:c r="D1" t="str">
-        <x:v>Evidence link</x:v>
-      </x:c>
-      <x:c r="E1" t="str">
-        <x:v>Notes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>G0 Charter</x:v>
-      </x:c>
-      <x:c r="B2" t="str"/>
-      <x:c r="C2" t="str"/>
-      <x:c r="D2" t="str"/>
-      <x:c r="E2" t="str"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>G1 Coordinate Lock</x:v>
-      </x:c>
-      <x:c r="B3" t="str"/>
-      <x:c r="C3" t="str"/>
-      <x:c r="D3" t="str"/>
-      <x:c r="E3" t="str"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>G2 Source Universe</x:v>
-      </x:c>
-      <x:c r="B4" t="str"/>
-      <x:c r="C4" t="str"/>
-      <x:c r="D4" t="str"/>
-      <x:c r="E4" t="str"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>G3 Row Integrity</x:v>
-      </x:c>
-      <x:c r="B5" t="str"/>
-      <x:c r="C5" t="str"/>
-      <x:c r="D5" t="str"/>
-      <x:c r="E5" t="str"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>G4 Dependence and Bias</x:v>
-      </x:c>
-      <x:c r="B6" t="str"/>
-      <x:c r="C6" t="str"/>
-      <x:c r="D6" t="str"/>
-      <x:c r="E6" t="str"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>G5 Statistical Method</x:v>
-      </x:c>
-      <x:c r="B7" t="str"/>
-      <x:c r="C7" t="str"/>
-      <x:c r="D7" t="str"/>
-      <x:c r="E7" t="str"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>G6 Reproducibility</x:v>
-      </x:c>
-      <x:c r="B8" t="str"/>
-      <x:c r="C8" t="str"/>
-      <x:c r="D8" t="str"/>
-      <x:c r="E8" t="str"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>G7 Release</x:v>
-      </x:c>
-      <x:c r="B9" t="str"/>
-      <x:c r="C9" t="str"/>
-      <x:c r="D9" t="str"/>
-      <x:c r="E9" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1310,6 +1571,104 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Gate</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>Evidence link</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>G0 Charter</x:v>
+      </x:c>
+      <x:c r="B2" t="str"/>
+      <x:c r="C2" t="str"/>
+      <x:c r="D2" t="str"/>
+      <x:c r="E2" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>G1 Coordinate Lock</x:v>
+      </x:c>
+      <x:c r="B3" t="str"/>
+      <x:c r="C3" t="str"/>
+      <x:c r="D3" t="str"/>
+      <x:c r="E3" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>G2 Source Universe</x:v>
+      </x:c>
+      <x:c r="B4" t="str"/>
+      <x:c r="C4" t="str"/>
+      <x:c r="D4" t="str"/>
+      <x:c r="E4" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>G3 Row Integrity</x:v>
+      </x:c>
+      <x:c r="B5" t="str"/>
+      <x:c r="C5" t="str"/>
+      <x:c r="D5" t="str"/>
+      <x:c r="E5" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>G4 Dependence and Bias</x:v>
+      </x:c>
+      <x:c r="B6" t="str"/>
+      <x:c r="C6" t="str"/>
+      <x:c r="D6" t="str"/>
+      <x:c r="E6" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>G5 Statistical Method</x:v>
+      </x:c>
+      <x:c r="B7" t="str"/>
+      <x:c r="C7" t="str"/>
+      <x:c r="D7" t="str"/>
+      <x:c r="E7" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>G6 Reproducibility</x:v>
+      </x:c>
+      <x:c r="B8" t="str"/>
+      <x:c r="C8" t="str"/>
+      <x:c r="D8" t="str"/>
+      <x:c r="E8" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>G7 Release</x:v>
+      </x:c>
+      <x:c r="B9" t="str"/>
+      <x:c r="C9" t="str"/>
+      <x:c r="D9" t="str"/>
+      <x:c r="E9" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -1473,13 +1832,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Regulatory and deployment</x:v>
+        <x:v>Trust maintenance</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>Safety supervisor review, audit, validation, training, regulated deployment</x:v>
+        <x:v>Checkpoint honesty, reliance positioning, trust debt, claim trace</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>supervisor packet, audit procedure, validation plan, training plan, regulated addendum, deployment playbook, 90-day roadmap</x:v>
+        <x:v>trust maintenance protocol, trust checkpoint map, trust positioning, trust status summary</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1487,12 +1846,26 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B13" t="str">
+        <x:v>Regulatory and deployment</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Safety supervisor review, audit, validation, training, regulated deployment</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>supervisor packet, audit procedure, validation plan, training plan, regulated addendum, deployment playbook, 90-day roadmap</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
         <x:v>Platform</x:v>
       </x:c>
-      <x:c r="C13" t="str">
+      <x:c r="C14" t="str">
         <x:v>Software workflow modules</x:v>
       </x:c>
-      <x:c r="D13" t="str">
+      <x:c r="D14" t="str">
         <x:v>future product layer</x:v>
       </x:c>
     </x:row>
@@ -1881,15 +2254,99 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
+        <x:v>TRUST-01</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Build ledger</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Track material work while package is being built</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>build_ledger.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>TRUST-02</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>Trust checkpoint review</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Prevent silent promotion of unchecked artifacts</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>checkpoint_reviews.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>TRUST-03</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>Assumption and uncertainty log</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Prevent assumptions becoming facts</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>assumption_uncertainty_log.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>TRUST-04</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>Claim trace matrix</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>Tie every claim to evidence, controls, gates, and permitted reliance</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>claim_trace_matrix.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>TRUST-05</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>Trust debt register</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>Track unresolved trust gaps with owner, due date, and release impact</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>trust_debt_register.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>TRUST-06</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>Reliance positioning</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>State what the package is trustworthy for and not trustworthy for</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>trust status summary, decision memo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
         <x:v>TRAIN-01</x:v>
       </x:c>
-      <x:c r="B20" t="str">
+      <x:c r="B26" t="str">
         <x:v>Role training</x:v>
       </x:c>
-      <x:c r="C20" t="str">
+      <x:c r="C26" t="str">
         <x:v>Ensure operators know controls</x:v>
       </x:c>
-      <x:c r="D20" t="str">
+      <x:c r="D26" t="str">
         <x:v>training matrix</x:v>
       </x:c>
     </x:row>
@@ -2463,12 +2920,23 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
+        <x:v>10_trust_maintenance</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>build ledger, checkpoints, assumptions, claim trace, trust debt</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>build_ledger.csv; checkpoint_reviews.csv; assumption_uncertainty_log.csv; claim_trace_matrix.csv; trust_debt_register.csv; trust_status_summary.md; open_questions.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
         <x:v>registers</x:v>
       </x:c>
-      <x:c r="B12" t="str">
+      <x:c r="B13" t="str">
         <x:v>package-level governance registers</x:v>
       </x:c>
-      <x:c r="C12" t="str">
+      <x:c r="C13" t="str">
         <x:v>document; control; gate; assurance; CAPA; decision; risk; training</x:v>
       </x:c>
     </x:row>

</xml_diff>